<commit_message>
Addition of course functionality + educational programme database
</commit_message>
<xml_diff>
--- a/_additional/alnas_xlsx/static/description/example/example.xlsx
+++ b/_additional/alnas_xlsx/static/description/example/example.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27628"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Imran Nas\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7CFA55-2F60-4666-834F-D1F22FD7AB4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{80227B3F-7A30-4C94-953A-8D3D36EC756B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="11016"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" calcOnSave="0"/>
+  <calcPr calcId="144525" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,15 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>Name</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
-    <t>Date</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Address</t>
     <phoneticPr fontId="0" type="noConversion"/>
@@ -42,36 +28,51 @@
     <t xml:space="preserve">   {%xv sysdate%}   </t>
   </si>
   <si>
-    <t>Report Sale Order {{docs.name}}</t>
-  </si>
-  <si>
     <t>{{docs.partner_id.name}}</t>
   </si>
   <si>
-    <t>{{docs.partner_id.contact_address_complete}}</t>
+    <t>{% endfor %}</t>
   </si>
   <si>
-    <t>{% for o in docs.order_line %}</t>
+    <t>Звіт з наявних баз проходження практик</t>
   </si>
   <si>
-    <t>{{o.price_subtotal}}</t>
+    <t>Сформовано:</t>
   </si>
   <si>
-    <t>Price Subtotal</t>
+    <t>Дата</t>
   </si>
   <si>
-    <t>Total = {{docs.amount_total}}</t>
+    <t>Список наявних баз практики</t>
   </si>
   <si>
-    <t>{% endfor %}</t>
+    <t>{% for line in docs.enterprises_ids %}</t>
+  </si>
+  <si>
+    <t>{{line.name}}</t>
+  </si>
+  <si>
+    <t>{{line.edrpou}}</t>
+  </si>
+  <si>
+    <t>{{line.adress}}</t>
+  </si>
+  <si>
+    <t>{{line.practise_type}}</t>
+  </si>
+  <si>
+    <t>{{line.partner_id.name}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="[$-409]d\-mmm\-yy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
   <fonts count="44">
     <font>
@@ -85,12 +86,6 @@
       <sz val="10"/>
       <name val="宋体"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color indexed="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="18"/>
@@ -403,6 +398,13 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="33">
@@ -756,209 +758,79 @@
   </borders>
   <cellStyleXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
@@ -968,79 +840,233 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1050,137 +1076,131 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="91">
-    <cellStyle name="20% - 强调文字颜色 1 2" xfId="2" xr:uid="{8CD2368A-ACD0-4A97-8DB2-121A11D8881F}"/>
-    <cellStyle name="20% - 强调文字颜色 1 2 2" xfId="46" xr:uid="{2ECEC457-576C-4560-9E45-08D3CEBD2526}"/>
-    <cellStyle name="20% - 强调文字颜色 2 2" xfId="3" xr:uid="{667B892C-8FB4-45EF-8639-17E8BF90F836}"/>
-    <cellStyle name="20% - 强调文字颜色 2 2 2" xfId="47" xr:uid="{50BED9A6-F88C-457E-917C-D33CC056CCF5}"/>
-    <cellStyle name="20% - 强调文字颜色 3 2" xfId="4" xr:uid="{47E725ED-BA9C-49C2-9690-5719E98C7C5F}"/>
-    <cellStyle name="20% - 强调文字颜色 3 2 2" xfId="48" xr:uid="{84B7BF93-737B-43C7-9749-5F414AE95F42}"/>
-    <cellStyle name="20% - 强调文字颜色 4 2" xfId="5" xr:uid="{A1AFCD5E-E0A0-4969-9D32-A24C161305AF}"/>
-    <cellStyle name="20% - 强调文字颜色 4 2 2" xfId="49" xr:uid="{80CCE9C7-01AA-45F4-BA6D-FC0657B7ACFC}"/>
-    <cellStyle name="20% - 强调文字颜色 5 2" xfId="6" xr:uid="{282B7947-9900-4BE3-B2DB-01854B92E55D}"/>
-    <cellStyle name="20% - 强调文字颜色 5 2 2" xfId="50" xr:uid="{C091D255-6D2C-4605-A936-8DA7D0BEA46D}"/>
-    <cellStyle name="20% - 强调文字颜色 6 2" xfId="7" xr:uid="{B6966BBF-2FCF-41B5-A9EE-54FC78B040FD}"/>
-    <cellStyle name="20% - 强调文字颜色 6 2 2" xfId="51" xr:uid="{0A3774C3-9E0A-432B-AE89-F3241AA7CAAF}"/>
-    <cellStyle name="40% - 强调文字颜色 1 2" xfId="8" xr:uid="{2327ECA8-AF2D-4200-83BD-C116DF590070}"/>
-    <cellStyle name="40% - 强调文字颜色 1 2 2" xfId="52" xr:uid="{4964A722-E38D-47AC-A671-D595598B429C}"/>
-    <cellStyle name="40% - 强调文字颜色 2 2" xfId="9" xr:uid="{4F77F814-662C-4563-8CA4-92ED54FC6737}"/>
-    <cellStyle name="40% - 强调文字颜色 2 2 2" xfId="53" xr:uid="{E011F25E-8FEA-4CF9-958E-876016D06A0E}"/>
-    <cellStyle name="40% - 强调文字颜色 3 2" xfId="10" xr:uid="{A7433C16-6EC6-4DA6-8464-2DFC6D8D392D}"/>
-    <cellStyle name="40% - 强调文字颜色 3 2 2" xfId="54" xr:uid="{AB8EB3C3-8E29-4B80-81E4-F01F9A010A5F}"/>
-    <cellStyle name="40% - 强调文字颜色 4 2" xfId="11" xr:uid="{FDCF99DE-DB56-405C-BD74-E7D9435B2B79}"/>
-    <cellStyle name="40% - 强调文字颜色 4 2 2" xfId="55" xr:uid="{D8CF32BD-A539-4275-994F-B72C4A4615E7}"/>
-    <cellStyle name="40% - 强调文字颜色 5 2" xfId="12" xr:uid="{4067F35A-0135-4AC0-BD75-733BCCB077E4}"/>
-    <cellStyle name="40% - 强调文字颜色 5 2 2" xfId="56" xr:uid="{0FE656C5-0603-4B91-9B0F-2876EEAF2045}"/>
-    <cellStyle name="40% - 强调文字颜色 6 2" xfId="13" xr:uid="{AED227D0-17CD-4F26-892D-546A1D701B42}"/>
-    <cellStyle name="40% - 强调文字颜色 6 2 2" xfId="57" xr:uid="{439B5303-7381-4C53-9290-022616067E1F}"/>
-    <cellStyle name="60% - 强调文字颜色 1 2" xfId="14" xr:uid="{5D4AE1C4-5B8B-4414-A3B4-FE4C531C9D04}"/>
-    <cellStyle name="60% - 强调文字颜色 1 2 2" xfId="58" xr:uid="{570306D6-8E46-414B-A63D-BD0098665BE0}"/>
-    <cellStyle name="60% - 强调文字颜色 2 2" xfId="15" xr:uid="{614BDBC3-4E7C-418A-B50B-EB3BD0C2C024}"/>
-    <cellStyle name="60% - 强调文字颜色 2 2 2" xfId="59" xr:uid="{AC5EED81-3C37-4C8A-93C3-5274649EA9DD}"/>
-    <cellStyle name="60% - 强调文字颜色 3 2" xfId="16" xr:uid="{38ADE76A-DAFE-4130-9551-7EE8F6360527}"/>
-    <cellStyle name="60% - 强调文字颜色 3 2 2" xfId="60" xr:uid="{EA092D81-4ADD-4F52-9BBF-4E1A41980C56}"/>
-    <cellStyle name="60% - 强调文字颜色 4 2" xfId="17" xr:uid="{3115415A-B9C1-4DE0-9E9F-9B887B2BD234}"/>
-    <cellStyle name="60% - 强调文字颜色 4 2 2" xfId="61" xr:uid="{A8E5E041-2A55-441C-A3DE-4C1378B5884C}"/>
-    <cellStyle name="60% - 强调文字颜色 5 2" xfId="18" xr:uid="{060B4C4B-BD44-4146-99AC-7EA51BF1B747}"/>
-    <cellStyle name="60% - 强调文字颜色 5 2 2" xfId="62" xr:uid="{3DB38FBC-C36D-4CD1-A700-9FEB9CB46473}"/>
-    <cellStyle name="60% - 强调文字颜色 6 2" xfId="19" xr:uid="{8E3DFE9B-5904-4D73-A96C-09702C71AC20}"/>
-    <cellStyle name="60% - 强调文字颜色 6 2 2" xfId="63" xr:uid="{46B7C93F-43C2-4CEB-A658-7F0A265D52DD}"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{9AC4454A-C689-4782-B6E0-5C0210581E16}"/>
-    <cellStyle name="好 2" xfId="29" xr:uid="{71285C49-D430-4D0C-AAC5-F674EB3278D8}"/>
-    <cellStyle name="好 2 2" xfId="73" xr:uid="{B5567CA2-83EA-49D0-814A-FC6AFCDED6E1}"/>
-    <cellStyle name="差 2" xfId="25" xr:uid="{5081DFBA-DD0D-4E6C-B643-C617EA4ED368}"/>
-    <cellStyle name="差 2 2" xfId="69" xr:uid="{FAB741BF-42CA-49C6-A835-A35D97BE1C9A}"/>
-    <cellStyle name="常规 2" xfId="26" xr:uid="{652BB157-1A51-43F6-B1BB-2ECBB5ED3A7B}"/>
-    <cellStyle name="常规 2 2" xfId="70" xr:uid="{15546EE3-28B0-4D9F-B306-266BFBD8B45C}"/>
-    <cellStyle name="常规 3" xfId="27" xr:uid="{B53A7ABD-901E-431B-9880-A1A5A1EF6276}"/>
-    <cellStyle name="常规 3 2" xfId="71" xr:uid="{920A0A79-491A-4434-9858-F3729FEC72FF}"/>
-    <cellStyle name="常规 4" xfId="28" xr:uid="{96564B52-BB1C-4F86-9C9E-5F43280DB2F1}"/>
-    <cellStyle name="常规 4 2" xfId="72" xr:uid="{9C2EE033-C216-4EC0-8AE0-7F92C121B589}"/>
-    <cellStyle name="常规 4 3" xfId="90" xr:uid="{4E242A86-790C-4B70-968B-0A13754F3B3F}"/>
-    <cellStyle name="强调文字颜色 1 2" xfId="36" xr:uid="{1C11B595-8E9B-4670-9E9C-4DA17789DE1F}"/>
-    <cellStyle name="强调文字颜色 1 2 2" xfId="80" xr:uid="{90A5ECE4-3807-4500-9F35-B7BBF79F9DB7}"/>
-    <cellStyle name="强调文字颜色 2 2" xfId="37" xr:uid="{E554994A-34D3-48F0-9D69-0C62806AEFA6}"/>
-    <cellStyle name="强调文字颜色 2 2 2" xfId="81" xr:uid="{0B6F0D1D-8502-4B26-AE3D-95425096A3AF}"/>
-    <cellStyle name="强调文字颜色 3 2" xfId="38" xr:uid="{4EA1C688-0589-4431-8D95-01DF8A9A0828}"/>
-    <cellStyle name="强调文字颜色 3 2 2" xfId="82" xr:uid="{679DED0A-98F6-4775-B9EA-913CF2CCE42F}"/>
-    <cellStyle name="强调文字颜色 4 2" xfId="39" xr:uid="{D13EF45D-E16D-4616-B0B2-C6DA0EA78F48}"/>
-    <cellStyle name="强调文字颜色 4 2 2" xfId="83" xr:uid="{D72C965F-37C5-448D-839A-A679B3722687}"/>
-    <cellStyle name="强调文字颜色 5 2" xfId="40" xr:uid="{02DC983E-99C9-4BFE-82D5-AF578725D3FD}"/>
-    <cellStyle name="强调文字颜色 5 2 2" xfId="84" xr:uid="{EFC9E413-880C-4978-B8EE-E5B45FF6245B}"/>
-    <cellStyle name="强调文字颜色 6 2" xfId="41" xr:uid="{40461524-C641-4398-983A-04AD892C28BC}"/>
-    <cellStyle name="强调文字颜色 6 2 2" xfId="85" xr:uid="{F0DB5463-CF4A-44DC-9805-1BE6D1895901}"/>
-    <cellStyle name="标题 1 2" xfId="20" xr:uid="{50F0BB1C-DF0E-4C23-A045-C9AD90E31727}"/>
-    <cellStyle name="标题 1 2 2" xfId="64" xr:uid="{032A3922-FB4A-4D2C-82F5-7048F99C3696}"/>
-    <cellStyle name="标题 2 2" xfId="21" xr:uid="{EA02FBB9-3033-4BA1-BF6E-F0E6ABFED573}"/>
-    <cellStyle name="标题 2 2 2" xfId="65" xr:uid="{A7F3C681-2799-4903-B87E-0BF527C62451}"/>
-    <cellStyle name="标题 3 2" xfId="22" xr:uid="{0CE91E1B-6652-4E76-B583-4018F4A19777}"/>
-    <cellStyle name="标题 3 2 2" xfId="66" xr:uid="{BE1D3408-BD21-45BD-92DF-E046EEA14011}"/>
-    <cellStyle name="标题 4 2" xfId="23" xr:uid="{25FB9BB7-35B0-4695-BAFF-88A05B436636}"/>
-    <cellStyle name="标题 4 2 2" xfId="67" xr:uid="{DD1B4389-EA46-4B1B-97BD-0E1D64574D97}"/>
-    <cellStyle name="标题 5" xfId="24" xr:uid="{638E2B53-BF43-4CF9-AB8C-FD2B9954245C}"/>
-    <cellStyle name="标题 5 2" xfId="68" xr:uid="{E5723CE8-9FF6-49E8-8975-8C0221D03D05}"/>
-    <cellStyle name="检查单元格 2" xfId="32" xr:uid="{E07B778F-F5B3-470D-828A-4F68ECDB24FC}"/>
-    <cellStyle name="检查单元格 2 2" xfId="76" xr:uid="{F6511D1D-1870-4E20-90C5-20070F86EC99}"/>
-    <cellStyle name="汇总 2" xfId="30" xr:uid="{C05FF64C-45F1-43CD-A879-7B36F7FF05DA}"/>
-    <cellStyle name="汇总 2 2" xfId="74" xr:uid="{5602C757-3611-4826-AE25-46A84B64718C}"/>
-    <cellStyle name="注释 2" xfId="45" xr:uid="{8859371A-6C49-4B67-BB70-D3C5F912AE9B}"/>
-    <cellStyle name="注释 2 2" xfId="89" xr:uid="{E53596B5-B437-4360-9BEA-9513864542F1}"/>
-    <cellStyle name="解释性文本 2" xfId="33" xr:uid="{ACED8140-ED47-4783-A5DF-210D620FA914}"/>
-    <cellStyle name="解释性文本 2 2" xfId="77" xr:uid="{827B898F-A58A-4733-A53E-74BF8910B47A}"/>
-    <cellStyle name="警告文本 2" xfId="34" xr:uid="{6705A38C-3802-4BFC-9A8D-7C2AA7A31FD4}"/>
-    <cellStyle name="警告文本 2 2" xfId="78" xr:uid="{4392691E-764A-4285-991F-8A0B0475A58F}"/>
-    <cellStyle name="计算 2" xfId="31" xr:uid="{7DFD60D9-D693-46E0-BEB7-5738F9E29F2C}"/>
-    <cellStyle name="计算 2 2" xfId="75" xr:uid="{03BAFD3B-8990-4C0E-8CC6-29A162DCA522}"/>
-    <cellStyle name="输入 2" xfId="44" xr:uid="{5CF57087-B3BD-40D3-9713-9A5CA848C326}"/>
-    <cellStyle name="输入 2 2" xfId="88" xr:uid="{306BF9B5-B6B6-4265-B9E2-ACC7EE92559A}"/>
-    <cellStyle name="输出 2" xfId="43" xr:uid="{E6EE602D-5C46-450E-8041-CD87FB538378}"/>
-    <cellStyle name="输出 2 2" xfId="87" xr:uid="{707B427B-1E13-4C96-B6C7-2F6527F741FB}"/>
-    <cellStyle name="适中 2" xfId="42" xr:uid="{D65C4771-F68A-41CB-BCF7-DA4193A70C17}"/>
-    <cellStyle name="适中 2 2" xfId="86" xr:uid="{A4949472-498F-48EB-83B5-496F2D05BB72}"/>
-    <cellStyle name="链接单元格 2" xfId="35" xr:uid="{4244553C-37EA-4B9D-9A1D-5FD65E7CD841}"/>
-    <cellStyle name="链接单元格 2 2" xfId="79" xr:uid="{3C5CD254-665C-490B-96E6-043467F9F689}"/>
+    <cellStyle name="20% - 强调文字颜色 1 2" xfId="2"/>
+    <cellStyle name="20% - 强调文字颜色 1 2 2" xfId="46"/>
+    <cellStyle name="20% - 强调文字颜色 2 2" xfId="3"/>
+    <cellStyle name="20% - 强调文字颜色 2 2 2" xfId="47"/>
+    <cellStyle name="20% - 强调文字颜色 3 2" xfId="4"/>
+    <cellStyle name="20% - 强调文字颜色 3 2 2" xfId="48"/>
+    <cellStyle name="20% - 强调文字颜色 4 2" xfId="5"/>
+    <cellStyle name="20% - 强调文字颜色 4 2 2" xfId="49"/>
+    <cellStyle name="20% - 强调文字颜色 5 2" xfId="6"/>
+    <cellStyle name="20% - 强调文字颜色 5 2 2" xfId="50"/>
+    <cellStyle name="20% - 强调文字颜色 6 2" xfId="7"/>
+    <cellStyle name="20% - 强调文字颜色 6 2 2" xfId="51"/>
+    <cellStyle name="40% - 强调文字颜色 1 2" xfId="8"/>
+    <cellStyle name="40% - 强调文字颜色 1 2 2" xfId="52"/>
+    <cellStyle name="40% - 强调文字颜色 2 2" xfId="9"/>
+    <cellStyle name="40% - 强调文字颜色 2 2 2" xfId="53"/>
+    <cellStyle name="40% - 强调文字颜色 3 2" xfId="10"/>
+    <cellStyle name="40% - 强调文字颜色 3 2 2" xfId="54"/>
+    <cellStyle name="40% - 强调文字颜色 4 2" xfId="11"/>
+    <cellStyle name="40% - 强调文字颜色 4 2 2" xfId="55"/>
+    <cellStyle name="40% - 强调文字颜色 5 2" xfId="12"/>
+    <cellStyle name="40% - 强调文字颜色 5 2 2" xfId="56"/>
+    <cellStyle name="40% - 强调文字颜色 6 2" xfId="13"/>
+    <cellStyle name="40% - 强调文字颜色 6 2 2" xfId="57"/>
+    <cellStyle name="60% - 强调文字颜色 1 2" xfId="14"/>
+    <cellStyle name="60% - 强调文字颜色 1 2 2" xfId="58"/>
+    <cellStyle name="60% - 强调文字颜色 2 2" xfId="15"/>
+    <cellStyle name="60% - 强调文字颜色 2 2 2" xfId="59"/>
+    <cellStyle name="60% - 强调文字颜色 3 2" xfId="16"/>
+    <cellStyle name="60% - 强调文字颜色 3 2 2" xfId="60"/>
+    <cellStyle name="60% - 强调文字颜色 4 2" xfId="17"/>
+    <cellStyle name="60% - 强调文字颜色 4 2 2" xfId="61"/>
+    <cellStyle name="60% - 强调文字颜色 5 2" xfId="18"/>
+    <cellStyle name="60% - 强调文字颜色 5 2 2" xfId="62"/>
+    <cellStyle name="60% - 强调文字颜色 6 2" xfId="19"/>
+    <cellStyle name="60% - 强调文字颜色 6 2 2" xfId="63"/>
+    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="好 2" xfId="29"/>
+    <cellStyle name="好 2 2" xfId="73"/>
+    <cellStyle name="差 2" xfId="25"/>
+    <cellStyle name="差 2 2" xfId="69"/>
+    <cellStyle name="常规 2" xfId="26"/>
+    <cellStyle name="常规 2 2" xfId="70"/>
+    <cellStyle name="常规 3" xfId="27"/>
+    <cellStyle name="常规 3 2" xfId="71"/>
+    <cellStyle name="常规 4" xfId="28"/>
+    <cellStyle name="常规 4 2" xfId="72"/>
+    <cellStyle name="常规 4 3" xfId="90"/>
+    <cellStyle name="强调文字颜色 1 2" xfId="36"/>
+    <cellStyle name="强调文字颜色 1 2 2" xfId="80"/>
+    <cellStyle name="强调文字颜色 2 2" xfId="37"/>
+    <cellStyle name="强调文字颜色 2 2 2" xfId="81"/>
+    <cellStyle name="强调文字颜色 3 2" xfId="38"/>
+    <cellStyle name="强调文字颜色 3 2 2" xfId="82"/>
+    <cellStyle name="强调文字颜色 4 2" xfId="39"/>
+    <cellStyle name="强调文字颜色 4 2 2" xfId="83"/>
+    <cellStyle name="强调文字颜色 5 2" xfId="40"/>
+    <cellStyle name="强调文字颜色 5 2 2" xfId="84"/>
+    <cellStyle name="强调文字颜色 6 2" xfId="41"/>
+    <cellStyle name="强调文字颜色 6 2 2" xfId="85"/>
+    <cellStyle name="标题 1 2" xfId="20"/>
+    <cellStyle name="标题 1 2 2" xfId="64"/>
+    <cellStyle name="标题 2 2" xfId="21"/>
+    <cellStyle name="标题 2 2 2" xfId="65"/>
+    <cellStyle name="标题 3 2" xfId="22"/>
+    <cellStyle name="标题 3 2 2" xfId="66"/>
+    <cellStyle name="标题 4 2" xfId="23"/>
+    <cellStyle name="标题 4 2 2" xfId="67"/>
+    <cellStyle name="标题 5" xfId="24"/>
+    <cellStyle name="标题 5 2" xfId="68"/>
+    <cellStyle name="检查单元格 2" xfId="32"/>
+    <cellStyle name="检查单元格 2 2" xfId="76"/>
+    <cellStyle name="汇总 2" xfId="30"/>
+    <cellStyle name="汇总 2 2" xfId="74"/>
+    <cellStyle name="注释 2" xfId="45"/>
+    <cellStyle name="注释 2 2" xfId="89"/>
+    <cellStyle name="解释性文本 2" xfId="33"/>
+    <cellStyle name="解释性文本 2 2" xfId="77"/>
+    <cellStyle name="警告文本 2" xfId="34"/>
+    <cellStyle name="警告文本 2 2" xfId="78"/>
+    <cellStyle name="计算 2" xfId="31"/>
+    <cellStyle name="计算 2 2" xfId="75"/>
+    <cellStyle name="输入 2" xfId="44"/>
+    <cellStyle name="输入 2 2" xfId="88"/>
+    <cellStyle name="输出 2" xfId="43"/>
+    <cellStyle name="输出 2 2" xfId="87"/>
+    <cellStyle name="适中 2" xfId="42"/>
+    <cellStyle name="适中 2 2" xfId="86"/>
+    <cellStyle name="链接单元格 2" xfId="35"/>
+    <cellStyle name="链接单元格 2 2" xfId="79"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1238,7 +1258,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1290,7 +1310,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1484,171 +1504,177 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12C576E8-B3C8-4C56-9A3F-29DB2AE511B5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H19"/>
-  <sheetFormatPr defaultColWidth="9.54296875" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9.5546875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="51.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="9" style="1" customWidth="1"/>
-    <col min="6" max="6" width="7.453125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.90625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="20.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.54296875" style="1"/>
+    <col min="6" max="6" width="8.88671875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.5546875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
     </row>
-    <row r="2" spans="1:8" ht="22.5">
-      <c r="B2" s="8" t="s">
+    <row r="2" spans="1:8" ht="22.8">
+      <c r="B2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
     </row>
-    <row r="3" spans="1:8" ht="15.5">
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
+    <row r="3" spans="1:8" ht="15">
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
     </row>
-    <row r="4" spans="1:8" ht="15.5" customHeight="1">
+    <row r="4" spans="1:8" ht="15.45" customHeight="1">
       <c r="B4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="10"/>
+    </row>
+    <row r="5" spans="1:8" ht="15">
+      <c r="B5" s="11"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="27.6">
+      <c r="B6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="19"/>
-    </row>
-    <row r="5" spans="1:8" ht="15.5">
-      <c r="B5" s="14"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15.5">
-      <c r="B6" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="13"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="20"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="B8" s="5" t="s">
-        <v>9</v>
+      <c r="B8" s="22" t="s">
+        <v>7</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="B9" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="26"/>
+      <c r="H9" s="27" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>10</v>
+      <c r="B10" s="7" t="s">
+        <v>14</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
     </row>
-    <row r="15" spans="1:8" ht="15">
-      <c r="A15" s="20"/>
+    <row r="15" spans="1:8" ht="15.6">
+      <c r="A15" s="5"/>
     </row>
-    <row r="16" spans="1:8" ht="15">
-      <c r="A16" s="21"/>
+    <row r="16" spans="1:8" ht="15.6">
+      <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:1" ht="15">
-      <c r="A17" s="21"/>
+    <row r="17" spans="1:1" ht="15.6">
+      <c r="A17" s="6"/>
     </row>
-    <row r="18" spans="1:1" ht="15">
-      <c r="A18" s="21"/>
+    <row r="18" spans="1:1" ht="15.6">
+      <c r="A18" s="6"/>
     </row>
-    <row r="19" spans="1:1" ht="15">
-      <c r="A19" s="20"/>
+    <row r="19" spans="1:1" ht="15.6">
+      <c r="A19" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="9">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="C6:H6"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="C4:H4"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B8:H8"/>
-    <mergeCell ref="B9:H9"/>
     <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="C6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>